<commit_message>
update in excel file
</commit_message>
<xml_diff>
--- a/excel file.xlsx
+++ b/excel file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/08f0634ad8470975/Documents/GitHub/CAP776-Daily-Work/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{6751269C-88D7-464F-BCF9-4CDEC4DB43DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E1E7A19-8908-4E12-AFB5-1EE3BA59D16F}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{6751269C-88D7-464F-BCF9-4CDEC4DB43DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66E505D8-48CB-4206-BF55-D0DD0137D5F6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="92">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -296,6 +296,12 @@
   </si>
   <si>
     <t>low</t>
+  </si>
+  <si>
+    <t>mumma is here today</t>
+  </si>
+  <si>
+    <t>travel back home</t>
   </si>
 </sst>
 </file>
@@ -2961,48 +2967,96 @@
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A47" s="8"/>
-      <c r="B47" s="9"/>
-      <c r="C47" s="9"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="9"/>
-      <c r="G47" s="9"/>
-      <c r="H47" s="9"/>
-      <c r="I47" s="15" t="str">
+      <c r="A47" s="8">
+        <v>46292</v>
+      </c>
+      <c r="B47" s="9">
+        <v>300</v>
+      </c>
+      <c r="C47" s="9">
+        <v>150</v>
+      </c>
+      <c r="D47" s="9">
+        <v>70</v>
+      </c>
+      <c r="E47" s="9">
+        <v>90</v>
+      </c>
+      <c r="F47" s="9">
+        <v>0</v>
+      </c>
+      <c r="G47" s="9">
+        <v>0</v>
+      </c>
+      <c r="H47" s="9">
+        <v>300</v>
+      </c>
+      <c r="I47" s="15">
         <f t="shared" si="4"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="J47" s="15" t="str">
+        <v>910</v>
+      </c>
+      <c r="J47" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K47" s="11"/>
-      <c r="L47" s="11"/>
-      <c r="M47" s="11"/>
-      <c r="N47" s="12"/>
+        <v>530</v>
+      </c>
+      <c r="K47" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L47" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M47" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="N47" s="12" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A48" s="8"/>
-      <c r="B48" s="9"/>
-      <c r="C48" s="9"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="9"/>
-      <c r="G48" s="9"/>
-      <c r="H48" s="9"/>
-      <c r="I48" s="15" t="str">
+      <c r="A48" s="8">
+        <v>46293</v>
+      </c>
+      <c r="B48" s="9">
+        <v>480</v>
+      </c>
+      <c r="C48" s="9">
+        <v>160</v>
+      </c>
+      <c r="D48" s="9">
+        <v>80</v>
+      </c>
+      <c r="E48" s="9">
+        <v>80</v>
+      </c>
+      <c r="F48" s="9">
+        <v>0</v>
+      </c>
+      <c r="G48" s="9">
+        <v>0</v>
+      </c>
+      <c r="H48" s="9">
+        <v>190</v>
+      </c>
+      <c r="I48" s="15">
         <f t="shared" si="4"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="J48" s="15" t="str">
+        <v>990</v>
+      </c>
+      <c r="J48" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K48" s="11"/>
-      <c r="L48" s="11"/>
-      <c r="M48" s="11"/>
-      <c r="N48" s="12"/>
+        <v>450</v>
+      </c>
+      <c r="K48" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L48" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="M48" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="N48" s="12" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="8"/>

</xml_diff>